<commit_message>
Delete SOP index 43 via Streamlit
</commit_message>
<xml_diff>
--- a/RCA.xlsx
+++ b/RCA.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J45"/>
+  <dimension ref="A1:J44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2746,50 +2746,6 @@
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" t="inlineStr"/>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>SYSTEM_FT</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>1111</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>Test bin</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>Test sub</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>Aass</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>Nooooooooo</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>無資料</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>無資料</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update SOP index 39 via Streamlit
</commit_message>
<xml_diff>
--- a/RCA.xlsx
+++ b/RCA.xlsx
@@ -2565,12 +2565,18 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>unknown issue</t>
+          <t>unknown issue (NV checking)</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>目前沒有解 (63865158400010)</t>
+          <t>1.Reseat the MGMT SSD on connector J41,. Confirm it is fully in the MGMT socket.
+2.Boot and check nvme list and lspci for the SSD. You want a device, link up, expected speed and width.
+3.If it is still missing, measure SSD power at the socket (3.3 V rail up after power-on) and confirm PERST is released (not held low).
+4.Swap the SSD with a unit that passed sbc_storage_ssd on the same station.
+o Fail follows the SSD: that drive or its PSID label.
+o Fail stays on the board: socket, SSD power enable, or PCIe (REFCLK / PERST / lane). Do not start with the CPU.
+Repeat the swap on one more of the four. If both follow the SSD, hold the lot and check the SSD date code before more rework</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">

</xml_diff>

<commit_message>
Add new SOP via Streamlit
</commit_message>
<xml_diff>
--- a/RCA.xlsx
+++ b/RCA.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J44"/>
+  <dimension ref="A1:J45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2752,6 +2752,50 @@
         </is>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="inlineStr"/>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>SYSTEM_FT</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>a6d70386</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>query_fnm_linkup-linkup_polling_fnm-FAIL-MEASUREMENT</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>linkup matrix_fnm-Failed:['port 65/0', 'port 65/1']</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>fnm issue ??</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>少見問題, 問題確認中</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>SN_63865158370022</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update SOP index 21 via Streamlit
</commit_message>
<xml_diff>
--- a/RCA.xlsx
+++ b/RCA.xlsx
@@ -1607,7 +1607,13 @@
         <is>
           <t>change the test stataion, NV will remove this test item ??
 Retest
-(客人說是超過70度的原因 但檢查溫度沒有看出來 目前這項軟體認為不需要在FT測試這個 他們會討論移除這個項目)</t>
+(客人說是超過70度的原因 但檢查溫度沒有看出來 目前這項軟體認為不需要在FT測試這個 他們會討論移除這個項目)
+若出現此相關
+CPLD mnb cpld main i2c, Register 2obf, bit hscl vin pg
+CPLD mnb cpld main i2c,Register 2oDf, bit hsc2 vin pg
+CPLD mnb cpld main i2c, Register 20E0, bit hsc3 vin pg
+CPLD mnb cpld main i2c, Register 2Eo, bit hsc4 vin pg
+--&gt;NV Eliko : put it aside</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1617,7 +1623,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>無資料</t>
+          <t>SN_63665152170002</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -2753,7 +2759,11 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr"/>
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
       <c r="B45" t="inlineStr">
         <is>
           <t>SYSTEM_FT</t>
@@ -2794,7 +2804,11 @@
           <t>SN_63865158370022</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr"/>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update SOP index 31 via Streamlit
</commit_message>
<xml_diff>
--- a/RCA.xlsx
+++ b/RCA.xlsx
@@ -2146,7 +2146,7 @@
 9.BMC有log, 停在check point 15 =&gt; 換MGMT, DDR (63465147980055)
 10.CPU console : Failed to start ntpsec.service =&gt; 測站問題 (TS2#69)
 11.CPU console : ONIE: OS Install Mode ... =&gt; SSD沒有燒 (TS1#51)
-12.Start PXE over IPv4.....目前沒有解 (63865158400049)</t>
+12.Start PXE over IPv4.....目前沒有解 (63865158400049)  --&gt;  Ahmad在解</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -2156,7 +2156,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>(TS2#89)</t>
+          <t>(TS2#89)(SN_63865158400049)</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">

</xml_diff>

<commit_message>
Update SOP index 6 via Streamlit
</commit_message>
<xml_diff>
--- a/RCA.xlsx
+++ b/RCA.xlsx
@@ -802,7 +802,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>csm_system-gpio-system_gpio_cplds-FAIL-MEASUREMENT</t>
+          <t>csm_system_gpio-system_gpio_cplds-FAIL-MEASUREMENT</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -2863,7 +2863,11 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr"/>
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
       <c r="B47" t="inlineStr">
         <is>
           <t>SYSTEM_FT</t>
@@ -2904,7 +2908,11 @@
           <t>無資料</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr"/>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update SOP index 20 via Streamlit
</commit_message>
<xml_diff>
--- a/RCA.xlsx
+++ b/RCA.xlsx
@@ -1551,9 +1551,9 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. if temperature = 100 then change test station (retest), still fail and then report case to TE
-2 .Remove the plastic gasket of WCK.
-3. Re-curing, re-assembly, change new WCK </t>
+          <t>1. if temperature = 100 then change test station (retest), still fail and then report case to TE
+2.Remove the plastic gasket of WCK.
+3. Re-curing, re-assembly, change new WCK</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2915,7 +2915,11 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr"/>
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
       <c r="B48" t="inlineStr">
         <is>
           <t>SYSTEM_FT</t>
@@ -2982,7 +2986,11 @@
           <t>TS1#34</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr"/>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update SOP index 45 via Streamlit
</commit_message>
<xml_diff>
--- a/RCA.xlsx
+++ b/RCA.xlsx
@@ -2895,7 +2895,8 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>TS1#34 已宣告不處理放棄
+6M 6-3 同樣問題，待宣告</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -2905,7 +2906,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>無資料</t>
+          <t>TS1#34(62865131330017)</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">

</xml_diff>

<commit_message>
Update SOP index 44 via Streamlit
</commit_message>
<xml_diff>
--- a/RCA.xlsx
+++ b/RCA.xlsx
@@ -2843,7 +2843,12 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>少見問題, 問題確認中</t>
+          <t>少見問題, 問題確認中
+1. 檢查QSFP是否有插好
+2. QSFP換一根試試
+3. 請ME開蓋檢查,QSFP cable是否有插好(重插拔一次)
+4. 檢查QSFP cable 接頭是否有問題(過去有發生頂針歪了)
+      --&gt; 需換QSFP cable</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -2994,7 +2999,11 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr"/>
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
       <c r="B49" t="inlineStr">
         <is>
           <t>MGMT_FT</t>
@@ -3035,7 +3044,11 @@
           <t>SN_63865158400010</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr"/>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>